<commit_message>
Related tdf#78486: propagate errors through calculated field references
When a calculated field referenced another field whose aggregated
result was in error state, the reference was silently replaced with
0.0, masking the upstream error. For example, with Field4 = '=2/0'
and Field5: "='Field4'/1", Field5 returned 0 instead of #VALUE!.

ReplaceTokenMeasuresWithValues now checks ScDPAggData::HasError()
after the inner calculation and emits a FormulaErrorToken on error
instead of a FormulaDoubleToken with the stale 0.0 fVal. The error
then propagates through the outer formula as #VALUE!, matching
Excel behavior and the already-correct =2/0 direct-error path.

Extend calcfields.xlsx / calcfields.xlsb fixtures with
Field5: "='Field4'/1"

Change-Id: Ibbd9af2b88eea913c362a892ece29fec1e0208e5
Reviewed-on: https://gerrit.libreoffice.org/c/core/+/204124
Tested-by: Jenkins
Reviewed-by: Balazs Varga <balazs.varga@collabora.com>
</commit_message>
<xml_diff>
--- a/sc/qa/unit/data/xlsx/pivot-table/calcfields.xlsx
+++ b/sc/qa/unit/data/xlsx/pivot-table/calcfields.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="15">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sum - Field4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum - Field5</t>
   </si>
   <si>
     <t xml:space="preserve">Total Result</t>
@@ -88,19 +91,16 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
     <font>
       <b val="true"/>
@@ -304,12 +304,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -361,6 +365,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -381,6 +389,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -390,6 +402,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -410,6 +426,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -444,7 +464,7 @@
   <cacheSource type="worksheet">
     <worksheetSource ref="J6:L24" sheet="Sheet1"/>
   </cacheSource>
-  <cacheFields count="7">
+  <cacheFields count="8">
     <cacheField name="Name" numFmtId="0">
       <sharedItems count="3">
         <s v="TATA"/>
@@ -471,8 +491,9 @@
     </cacheField>
     <cacheField name="Field1" numFmtId="0" formula="'Field A'*20" databaseField="0"/>
     <cacheField name="Field2" numFmtId="0" formula="SUM('Field A', 'Field B')" databaseField="0"/>
-    <cacheField name="Field3" numFmtId="0" formula="Name*2" databaseField="0"/>
-    <cacheField name="Field4" numFmtId="0" formula=" 2/0" databaseField="0"/>
+    <cacheField name="Field3" numFmtId="0" formula="'Name'*2" databaseField="0"/>
+    <cacheField name="Field4" numFmtId="0" formula="2/0" databaseField="0"/>
+    <cacheField name="Field5" numFmtId="0" formula=" 'Field4'/1" databaseField="0"/>
   </cacheFields>
 </pivotCacheDefinition>
 </file>
@@ -574,8 +595,8 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DataPilot1" cacheId="1" dataOnRows="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" showDrill="0" useAutoFormatting="0" itemPrintTitles="1" indent="0" outline="0" outlineData="0" compact="0" compactData="0">
-  <location ref="A1:G6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="7">
+  <location ref="A1:H6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="8">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -585,6 +606,7 @@
     </pivotField>
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -610,7 +632,8 @@
   <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="6">
+  <colItems count="7">
+    <i/>
     <i/>
     <i/>
     <i/>
@@ -618,13 +641,14 @@
     <i/>
     <i/>
   </colItems>
-  <dataFields count="6">
+  <dataFields count="7">
     <dataField name="Sum - Field A" fld="1" subtotal="sum" numFmtId="164"/>
     <dataField name="Sum - Field B" fld="2" subtotal="sum" numFmtId="165"/>
     <dataField name="Sum - Field1" fld="3" subtotal="sum" numFmtId="164"/>
     <dataField name="Sum - Field2" fld="4" subtotal="sum" numFmtId="164"/>
     <dataField name="Sum - Field3" fld="5" subtotal="sum" numFmtId="164"/>
     <dataField name="Sum - Field4" fld="6" subtotal="sum" numFmtId="164"/>
+    <dataField name="Sum - Field5" fld="7" subtotal="sum" numFmtId="164"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -811,211 +835,211 @@
   <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J6" s="0" t="s">
+      <c r="J6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="L6" s="0" t="s">
+      <c r="K6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J7" s="0" t="s">
+      <c r="J7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1" t="n">
+      <c r="K7" s="1">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J8" s="0" t="s">
+      <c r="J8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="1" t="n">
+      <c r="K8" s="1">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J9" s="0" t="s">
+      <c r="J9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K9" s="0" t="n">
+      <c r="K9" s="1">
         <v>5</v>
       </c>
-      <c r="L9" s="1" t="n">
+      <c r="L9" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J10" s="0" t="s">
+      <c r="J10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K10" s="0" t="n">
+      <c r="K10" s="1">
         <v>2</v>
       </c>
-      <c r="L10" s="1" t="n">
+      <c r="L10" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J11" s="0" t="s">
+      <c r="J11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K11" s="0" t="n">
+      <c r="K11" s="1">
         <v>12</v>
       </c>
-      <c r="L11" s="1" t="n">
+      <c r="L11" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J12" s="0" t="s">
+      <c r="J12" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K12" s="0" t="n">
+      <c r="K12" s="1">
         <v>3</v>
       </c>
-      <c r="L12" s="1" t="n">
+      <c r="L12" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J13" s="0" t="s">
+      <c r="J13" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K13" s="0" t="n">
+      <c r="K13" s="1">
         <v>5</v>
       </c>
-      <c r="L13" s="1" t="n">
+      <c r="L13" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J14" s="0" t="s">
+      <c r="J14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K14" s="0" t="n">
+      <c r="K14" s="1">
         <v>0</v>
       </c>
-      <c r="L14" s="1" t="n">
+      <c r="L14" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J15" s="0" t="s">
+      <c r="J15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K15" s="0" t="n">
+      <c r="K15" s="1">
         <v>3</v>
       </c>
-      <c r="L15" s="1" t="n">
+      <c r="L15" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J16" s="0" t="s">
+      <c r="J16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K16" s="0" t="n">
+      <c r="K16" s="1">
         <v>5</v>
       </c>
-      <c r="L16" s="1" t="n">
+      <c r="L16" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J17" s="0" t="s">
+      <c r="J17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K17" s="0" t="n">
+      <c r="K17" s="1">
         <v>9</v>
       </c>
-      <c r="L17" s="1" t="n">
+      <c r="L17" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J18" s="0" t="s">
+      <c r="J18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K18" s="0" t="n">
+      <c r="K18" s="1">
         <v>5</v>
       </c>
-      <c r="L18" s="1" t="n">
+      <c r="L18" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J19" s="0" t="s">
+      <c r="J19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K19" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="1" t="n">
+      <c r="K19" s="1">
+        <v>1</v>
+      </c>
+      <c r="L19" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J20" s="0" t="s">
+      <c r="J20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="1" t="n">
+      <c r="K20" s="1">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J21" s="0" t="s">
+      <c r="J21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" s="1" t="n">
+      <c r="K21" s="1">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J22" s="0" t="s">
+      <c r="J22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K22" s="0" t="n">
+      <c r="K22" s="1">
         <v>2</v>
       </c>
-      <c r="L22" s="1" t="n">
+      <c r="L22" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J23" s="0" t="s">
+      <c r="J23" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K23" s="0" t="n">
+      <c r="K23" s="1">
         <v>3</v>
       </c>
-      <c r="L23" s="1" t="n">
+      <c r="L23" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J24" s="0" t="s">
+      <c r="J24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K24" s="0" t="n">
+      <c r="K24" s="1">
         <v>55</v>
       </c>
-      <c r="L24" s="1" t="n">
+      <c r="L24" s="2">
         <v>1</v>
       </c>
     </row>
@@ -1035,135 +1059,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="12.78125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3"/>
+      <c r="B1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
       <c r="G1" s="5"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>12</v>
       </c>
+      <c r="H2" s="10" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="11" t="n">
+      <c r="B3" s="12">
         <v>24</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="13">
         <v>6</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="14">
         <v>480</v>
       </c>
-      <c r="E3" s="13" t="n">
+      <c r="E3" s="14">
         <v>30</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="14">
         <v>0</v>
       </c>
-      <c r="G3" s="14" t="e">
+      <c r="G3" s="15" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="C4" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" s="18" t="n">
-        <v>640</v>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>42</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="19" t="e">
+      <c r="H3" s="16" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>58</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>1160</v>
-      </c>
-      <c r="E5" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" s="22" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="18">
+        <v>32</v>
+      </c>
+      <c r="C4" s="19">
+        <v>10</v>
+      </c>
+      <c r="D4" s="20">
+        <v>640</v>
+      </c>
+      <c r="E4" s="20">
+        <v>42</v>
+      </c>
+      <c r="F4" s="20">
         <v>0</v>
       </c>
-      <c r="G5" s="23" t="e">
+      <c r="G4" s="21" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
+      <c r="H4" s="22" t="e">
+        <f aca="false">#VALUE!</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="23">
+        <v>58</v>
+      </c>
+      <c r="C5" s="24">
+        <v>2</v>
+      </c>
+      <c r="D5" s="25">
+        <v>1160</v>
+      </c>
+      <c r="E5" s="25">
+        <v>60</v>
+      </c>
+      <c r="F5" s="25">
+        <v>0</v>
+      </c>
+      <c r="G5" s="26" t="e">
+        <f aca="false">#VALUE!</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H5" s="27" t="e">
+        <f aca="false">#VALUE!</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="25" t="n">
+      <c r="A6" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="29">
         <v>114</v>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="30">
         <v>18</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="31">
         <v>2280</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="31">
         <v>132</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="31">
         <v>0</v>
       </c>
-      <c r="G6" s="28" t="e">
+      <c r="G6" s="32" t="e">
+        <f aca="false">#VALUE!</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H6" s="33" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>

</xml_diff>